<commit_message>
Update calendar and Champions League data files
Refreshed calendar.xlsx and championsLeagueRounds_24_25.xlsx with new or corrected data to ensure up-to-date scheduling and match information.
</commit_message>
<xml_diff>
--- a/past seasons data/championsLeagueRounds_24_25.xlsx
+++ b/past seasons data/championsLeagueRounds_24_25.xlsx
@@ -1,25 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acer\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ibram\OneDrive\Documents\GitHub\Egyptian-Premier-League-Schedule-Optimizer\past seasons data\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A31F2C-157B-43E5-B5D9-C7E31ABC318E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9264"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="استخراج جدول مواعيد جولات المبا" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="36">
   <si>
     <t>Round Name</t>
   </si>
@@ -76,17 +91,68 @@
   </si>
   <si>
     <t xml:space="preserve">End Date </t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>16/08/2024</t>
+  </si>
+  <si>
+    <t>17/08/2024</t>
+  </si>
+  <si>
+    <t>18/08/2024</t>
+  </si>
+  <si>
+    <t>23/08/2024</t>
+  </si>
+  <si>
+    <t>24/08/2024</t>
+  </si>
+  <si>
+    <t>25/08/2024</t>
+  </si>
+  <si>
+    <t>13/09/2024</t>
+  </si>
+  <si>
+    <t>14/09/2024</t>
+  </si>
+  <si>
+    <t>15/09/2024</t>
+  </si>
+  <si>
+    <t>20/09/2024</t>
+  </si>
+  <si>
+    <t>21/09/2024</t>
+  </si>
+  <si>
+    <t>22/09/2024</t>
+  </si>
+  <si>
+    <t>26/11/2024</t>
+  </si>
+  <si>
+    <t>19/04/2025</t>
+  </si>
+  <si>
+    <t>25/04/2025</t>
+  </si>
+  <si>
+    <t>24/05/2025</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -100,6 +166,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -109,7 +190,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -117,16 +198,39 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+  <cellXfs count="7">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -142,10 +246,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -345,201 +445,464 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:C17"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.44140625" customWidth="1"/>
+    <col min="1" max="1" width="22.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <v>45520</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="2">
         <v>45522</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>45527</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>45529</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>45548</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>45550</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>45555</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <v>45557</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>45520</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <v>45522</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="2">
         <v>45527</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="2">
         <v>45529</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="2">
         <v>45548</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="2">
         <v>45550</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="2">
         <v>45555</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="2">
         <v>45557</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="3">
         <v>45622</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="3">
         <v>45622</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="2">
         <v>45632</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="2">
         <v>45634</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" s="2">
         <v>45748</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="2">
         <v>45748</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="3">
+      <c r="B13" s="2">
         <v>45755</v>
       </c>
-      <c r="C13" s="3">
+      <c r="C13" s="2">
         <v>45756</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="3">
+      <c r="B14" s="2">
         <v>45766</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="2">
         <v>45766</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B15" s="2">
         <v>45772</v>
       </c>
-      <c r="C15" s="3">
+      <c r="C15" s="2">
         <v>45772</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B16" s="2">
         <v>45801</v>
       </c>
-      <c r="C16" s="3">
+      <c r="C16" s="2">
         <v>45801</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="3">
+      <c r="B17" s="2">
         <v>45809</v>
       </c>
-      <c r="C17" s="3">
+      <c r="C17" s="2">
         <v>45809</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{186521C1-DEDE-4739-A7C0-AFC26334477F}">
+  <dimension ref="A1:B36"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="9.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5"/>
+      <c r="B4" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5"/>
+      <c r="B6" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5"/>
+      <c r="B7" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="5"/>
+      <c r="B9" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="5"/>
+      <c r="B10" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="5"/>
+      <c r="B13" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="53.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="5"/>
+      <c r="B15" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="5"/>
+      <c r="B16" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="53.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="53.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="53.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="5"/>
+      <c r="B25" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="53.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="53.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B27" s="6">
+        <v>45455</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="5"/>
+      <c r="B28" s="6">
+        <v>45485</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="5"/>
+      <c r="B29" s="6">
+        <v>45516</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B30" s="6">
+        <v>45661</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31" s="6">
+        <v>45873</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="5"/>
+      <c r="B32" s="6">
+        <v>45904</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B36" s="6">
+        <v>45663</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modify dates for CAF
</commit_message>
<xml_diff>
--- a/past seasons data/championsLeagueRounds_24_25.xlsx
+++ b/past seasons data/championsLeagueRounds_24_25.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ibram\OneDrive\Documents\GitHub\Egyptian-Premier-League-Schedule-Optimizer\past seasons data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\Egyptian-Premier-League-Schedule-Optimizer\past seasons data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A31F2C-157B-43E5-B5D9-C7E31ABC318E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A5884CF-5591-4CB3-AC16-E885691AFBCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="استخراج جدول مواعيد جولات المبا" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="24">
   <si>
     <t>Round Name</t>
   </si>
@@ -96,52 +96,16 @@
     <t>Date</t>
   </si>
   <si>
-    <t>16/08/2024</t>
-  </si>
-  <si>
-    <t>17/08/2024</t>
-  </si>
-  <si>
-    <t>18/08/2024</t>
-  </si>
-  <si>
-    <t>23/08/2024</t>
-  </si>
-  <si>
-    <t>24/08/2024</t>
-  </si>
-  <si>
-    <t>25/08/2024</t>
-  </si>
-  <si>
-    <t>13/09/2024</t>
-  </si>
-  <si>
-    <t>14/09/2024</t>
-  </si>
-  <si>
-    <t>15/09/2024</t>
-  </si>
-  <si>
-    <t>20/09/2024</t>
-  </si>
-  <si>
-    <t>21/09/2024</t>
-  </si>
-  <si>
-    <t>22/09/2024</t>
-  </si>
-  <si>
-    <t>26/11/2024</t>
-  </si>
-  <si>
-    <t>19/04/2025</t>
-  </si>
-  <si>
-    <t>25/04/2025</t>
-  </si>
-  <si>
-    <t>24/05/2025</t>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>day</t>
+  </si>
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>year</t>
   </si>
 </sst>
 </file>
@@ -152,7 +116,7 @@
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -177,6 +141,19 @@
       <b/>
       <sz val="10"/>
       <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -217,7 +194,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -225,12 +202,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -515,10 +494,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="2">
-        <v>45520</v>
+        <v>45622</v>
       </c>
       <c r="C6" s="2">
-        <v>45522</v>
+        <v>45622</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
@@ -526,10 +505,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="2">
-        <v>45527</v>
+        <v>45632</v>
       </c>
       <c r="C7" s="2">
-        <v>45529</v>
+        <v>45634</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="13.2" x14ac:dyDescent="0.25">
@@ -649,263 +628,701 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{186521C1-DEDE-4739-A7C0-AFC26334477F}">
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="2" max="2" width="29.88671875" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C1" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="5">
+        <v>45520</v>
+      </c>
+      <c r="C2">
+        <f>DAY(B2)</f>
+        <v>16</v>
+      </c>
+      <c r="D2">
+        <f>MONTH(B2)</f>
+        <v>8</v>
+      </c>
+      <c r="E2">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="5">
+        <v>45520</v>
+      </c>
+      <c r="C3">
+        <f>DAY(B3)</f>
+        <v>16</v>
+      </c>
+      <c r="D3">
+        <f>MONTH(B3)</f>
+        <v>8</v>
+      </c>
+      <c r="E3">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="5">
+        <v>45521</v>
+      </c>
+      <c r="C4">
+        <f>DAY(B4)</f>
+        <v>17</v>
+      </c>
+      <c r="D4">
+        <f>MONTH(B4)</f>
+        <v>8</v>
+      </c>
+      <c r="E4">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="5">
+        <v>45521</v>
+      </c>
+      <c r="C5">
+        <f>DAY(B5)</f>
+        <v>17</v>
+      </c>
+      <c r="D5">
+        <f>MONTH(B5)</f>
+        <v>8</v>
+      </c>
+      <c r="E5">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="5">
+        <v>45522</v>
+      </c>
+      <c r="C6">
+        <f>DAY(B6)</f>
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <f>MONTH(B6)</f>
+        <v>8</v>
+      </c>
+      <c r="E6">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="5">
+        <v>45522</v>
+      </c>
+      <c r="C7">
+        <f>DAY(B7)</f>
+        <v>18</v>
+      </c>
+      <c r="D7">
+        <f>MONTH(B7)</f>
+        <v>8</v>
+      </c>
+      <c r="E7">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="5">
+        <v>45527</v>
+      </c>
+      <c r="C8">
+        <f>DAY(B8)</f>
+        <v>23</v>
+      </c>
+      <c r="D8">
+        <f>MONTH(B8)</f>
+        <v>8</v>
+      </c>
+      <c r="E8">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="5">
+        <v>45527</v>
+      </c>
+      <c r="C9">
+        <f>DAY(B9)</f>
+        <v>23</v>
+      </c>
+      <c r="D9">
+        <f>MONTH(B9)</f>
+        <v>8</v>
+      </c>
+      <c r="E9">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="5">
+        <v>45528</v>
+      </c>
+      <c r="C10">
+        <f>DAY(B10)</f>
+        <v>24</v>
+      </c>
+      <c r="D10">
+        <f>MONTH(B10)</f>
+        <v>8</v>
+      </c>
+      <c r="E10">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="5">
+        <v>45528</v>
+      </c>
+      <c r="C11">
+        <f>DAY(B11)</f>
+        <v>24</v>
+      </c>
+      <c r="D11">
+        <f>MONTH(B11)</f>
+        <v>8</v>
+      </c>
+      <c r="E11">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" s="5">
+        <v>45529</v>
+      </c>
+      <c r="C12">
+        <f>DAY(B12)</f>
+        <v>25</v>
+      </c>
+      <c r="D12">
+        <f>MONTH(B12)</f>
+        <v>8</v>
+      </c>
+      <c r="E12">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B13" s="5">
+        <v>45529</v>
+      </c>
+      <c r="C13">
+        <f>DAY(B13)</f>
+        <v>25</v>
+      </c>
+      <c r="D13">
+        <f>MONTH(B13)</f>
+        <v>8</v>
+      </c>
+      <c r="E13">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="5">
+        <v>45548</v>
+      </c>
+      <c r="C14">
+        <f>DAY(B14)</f>
+        <v>13</v>
+      </c>
+      <c r="D14">
+        <f>MONTH(B14)</f>
+        <v>9</v>
+      </c>
+      <c r="E14">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" s="5">
+        <v>45548</v>
+      </c>
+      <c r="C15">
+        <f>DAY(B15)</f>
+        <v>13</v>
+      </c>
+      <c r="D15">
+        <f>MONTH(B15)</f>
+        <v>9</v>
+      </c>
+      <c r="E15">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="5">
+        <v>45549</v>
+      </c>
+      <c r="C16">
+        <f>DAY(B16)</f>
+        <v>14</v>
+      </c>
+      <c r="D16">
+        <f>MONTH(B16)</f>
+        <v>9</v>
+      </c>
+      <c r="E16">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" s="5">
+        <v>45549</v>
+      </c>
+      <c r="C17">
+        <f>DAY(B17)</f>
+        <v>14</v>
+      </c>
+      <c r="D17">
+        <f>MONTH(B17)</f>
+        <v>9</v>
+      </c>
+      <c r="E17">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" s="5">
+        <v>45550</v>
+      </c>
+      <c r="C18">
+        <f>DAY(B18)</f>
+        <v>15</v>
+      </c>
+      <c r="D18">
+        <f>MONTH(B18)</f>
+        <v>9</v>
+      </c>
+      <c r="E18">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19" s="5">
+        <v>45550</v>
+      </c>
+      <c r="C19">
+        <f>DAY(B19)</f>
+        <v>15</v>
+      </c>
+      <c r="D19">
+        <f>MONTH(B19)</f>
+        <v>9</v>
+      </c>
+      <c r="E19">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" s="5">
+        <v>45555</v>
+      </c>
+      <c r="C20">
+        <f>DAY(B20)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5" t="s">
+      <c r="D20">
+        <f>MONTH(B20)</f>
+        <v>9</v>
+      </c>
+      <c r="E20">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B21" s="5">
+        <v>45555</v>
+      </c>
+      <c r="C21">
+        <f>DAY(B21)</f>
+        <v>20</v>
+      </c>
+      <c r="D21">
+        <f>MONTH(B21)</f>
+        <v>9</v>
+      </c>
+      <c r="E21">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22" s="5">
+        <v>45556</v>
+      </c>
+      <c r="C22">
+        <f>DAY(B22)</f>
         <v>21</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5" t="s">
+      <c r="D22">
+        <f>MONTH(B22)</f>
+        <v>9</v>
+      </c>
+      <c r="E22">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B23" s="5">
+        <v>45556</v>
+      </c>
+      <c r="C23">
+        <f>DAY(B23)</f>
+        <v>21</v>
+      </c>
+      <c r="D23">
+        <f>MONTH(B23)</f>
+        <v>9</v>
+      </c>
+      <c r="E23">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B24" s="5">
+        <v>45557</v>
+      </c>
+      <c r="C24">
+        <f>DAY(B24)</f>
         <v>22</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="5" t="s">
+      <c r="D24">
+        <f>MONTH(B24)</f>
+        <v>9</v>
+      </c>
+      <c r="E24">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B25" s="5">
+        <v>45557</v>
+      </c>
+      <c r="C25">
+        <f>DAY(B25)</f>
+        <v>22</v>
+      </c>
+      <c r="D25">
+        <f>MONTH(B25)</f>
+        <v>9</v>
+      </c>
+      <c r="E25">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26" s="5">
+        <v>45622</v>
+      </c>
+      <c r="C26">
+        <f>DAY(B26)</f>
         <v>26</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="53.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="53.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="53.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="5"/>
-      <c r="B22" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="53.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="5"/>
-      <c r="B24" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="5"/>
-      <c r="B25" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="53.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="53.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D26">
+        <f>MONTH(B26)</f>
+        <v>11</v>
+      </c>
+      <c r="E26">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B27" s="6">
-        <v>45455</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="5"/>
-      <c r="B28" s="6">
-        <v>45485</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="5"/>
-      <c r="B29" s="6">
-        <v>45516</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="5">
+        <v>45632</v>
+      </c>
+      <c r="C27">
+        <f>DAY(B27)</f>
+        <v>6</v>
+      </c>
+      <c r="D27">
+        <f>MONTH(B27)</f>
+        <v>12</v>
+      </c>
+      <c r="E27">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B28" s="5">
+        <v>45633</v>
+      </c>
+      <c r="C28">
+        <f>DAY(B28)</f>
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <f>MONTH(B28)</f>
+        <v>12</v>
+      </c>
+      <c r="E28">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B29" s="5">
+        <v>45634</v>
+      </c>
+      <c r="C29">
+        <f>DAY(B29)</f>
+        <v>8</v>
+      </c>
+      <c r="D29">
+        <f>MONTH(B29)</f>
+        <v>12</v>
+      </c>
+      <c r="E29">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B30" s="6">
-        <v>45661</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="5">
+        <v>45748</v>
+      </c>
+      <c r="C30">
+        <f>DAY(B30)</f>
+        <v>1</v>
+      </c>
+      <c r="D30">
+        <f>MONTH(B30)</f>
+        <v>4</v>
+      </c>
+      <c r="E30">
+        <v>2027</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B31" s="6">
-        <v>45873</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="5"/>
-      <c r="B32" s="6">
-        <v>45904</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="5">
+        <v>45755</v>
+      </c>
+      <c r="C31">
+        <f>DAY(B31)</f>
+        <v>8</v>
+      </c>
+      <c r="D31">
+        <f>MONTH(B31)</f>
+        <v>4</v>
+      </c>
+      <c r="E31">
+        <v>2027</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B32" s="5">
+        <v>45756</v>
+      </c>
+      <c r="C32">
+        <f>DAY(B32)</f>
+        <v>9</v>
+      </c>
+      <c r="D32">
+        <f>MONTH(B32)</f>
+        <v>4</v>
+      </c>
+      <c r="E32">
+        <v>2027</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B33" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="5">
+        <v>45766</v>
+      </c>
+      <c r="C33">
+        <f>DAY(B33)</f>
+        <v>19</v>
+      </c>
+      <c r="D33">
+        <f>MONTH(B33)</f>
+        <v>4</v>
+      </c>
+      <c r="E33">
+        <v>2027</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B34" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="5">
+        <v>45772</v>
+      </c>
+      <c r="C34">
+        <f>DAY(B34)</f>
+        <v>25</v>
+      </c>
+      <c r="D34">
+        <f>MONTH(B34)</f>
+        <v>4</v>
+      </c>
+      <c r="E34">
+        <v>2027</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B35" s="5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="5">
+        <v>45801</v>
+      </c>
+      <c r="C35">
+        <f>DAY(B35)</f>
+        <v>24</v>
+      </c>
+      <c r="D35">
+        <f>MONTH(B35)</f>
+        <v>5</v>
+      </c>
+      <c r="E35">
+        <v>2027</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B36" s="6">
-        <v>45663</v>
+      <c r="B36" s="5">
+        <v>45809</v>
+      </c>
+      <c r="C36">
+        <f>DAY(B36)</f>
+        <v>1</v>
+      </c>
+      <c r="D36">
+        <f>MONTH(B36)</f>
+        <v>6</v>
+      </c>
+      <c r="E36">
+        <v>2027</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E36">
+    <sortCondition ref="B1:B36"/>
+  </sortState>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>